<commit_message>
data(mt_gt): refresh employee/customer master data and GT ads cost
- Update "Nhân Viên.xlsx" and "khách hàng.xlsx" master data exports.
- ads.csv: replace stale 13/07/2026 row with GT ads cost for
  01-02/10/2026.
- Add CU.csv with GT ads cost history for 01/08-30/09/2026.

NOTE: mt_gt_etl.py detects ads master files by filename keyword
("ads"/"quảng cáo"/"chi phí"), not by exact name. "CU.csv" does not
match that pattern today, so the Aug-Sep GT ads data in it will NOT be
picked up by the ETL as-is — flagging for the user to confirm whether
it should be renamed/merged into ads.csv.
</commit_message>
<xml_diff>
--- a/data/mt_gt/2_master_data/Nhân Viên.xlsx
+++ b/data/mt_gt/2_master_data/Nhân Viên.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
   <si>
     <t>mã</t>
   </si>
@@ -52,6 +52,18 @@
   <si>
     <t>NV103</t>
   </si>
+  <si>
+    <t>NV044-HCM</t>
+  </si>
+  <si>
+    <t>NV0106</t>
+  </si>
+  <si>
+    <t>NV001</t>
+  </si>
+  <si>
+    <t>NV0108</t>
+  </si>
 </sst>
 </file>
 
@@ -63,13 +75,19 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -410,12 +428,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -536,139 +569,142 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1195,8 +1231,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="1"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1235,6 +1271,38 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>